<commit_message>
fix(literature): minor update to overview file
</commit_message>
<xml_diff>
--- a/05-rapid-literature-review/literature_review_overview.xlsx
+++ b/05-rapid-literature-review/literature_review_overview.xlsx
@@ -1,20 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Tim/Developer/MAST Dev/2026-10 ICSME Data Analysis Support/data-analysis-support/06-rapid-literature-review/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Tim/Developer/MAST Dev/2026-10 ICSME Data Analysis Support/data-agent-rep-pack/05-rapid-literature-review/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{520EAB6C-B2B9-A44A-86F1-D878449E2894}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F2C8E7C-6B3F-D44E-A653-6A54FE8A5C09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{17F07385-D941-E342-B840-EC6232492BEC}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17740" xr2:uid="{17F07385-D941-E342-B840-EC6232492BEC}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview Articles" sheetId="1" r:id="rId1"/>
-    <sheet name="Extracted Requirements" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Overview Articles'!$A$1:$L$1</definedName>
@@ -13695,56 +13694,4 @@
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82528CF6-6712-614D-8C42-14A8D71CE4B3}">
-  <dimension ref="A1:A321"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A1" s="1"/>
-    </row>
-    <row r="308" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A308" s="1"/>
-    </row>
-    <row r="309" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A309" s="1"/>
-    </row>
-    <row r="310" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A310" s="1"/>
-    </row>
-    <row r="311" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A311" s="2"/>
-    </row>
-    <row r="312" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A312" s="1"/>
-    </row>
-    <row r="314" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A314" s="1"/>
-    </row>
-    <row r="315" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A315" s="1"/>
-    </row>
-    <row r="316" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A316" s="1"/>
-    </row>
-    <row r="317" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A317" s="1"/>
-    </row>
-    <row r="318" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A318" s="1"/>
-    </row>
-    <row r="319" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A319" s="1"/>
-    </row>
-    <row r="320" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A320" s="2"/>
-    </row>
-    <row r="321" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A321" s="1"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>